<commit_message>
Align code with the architecture
</commit_message>
<xml_diff>
--- a/Docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/Docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,21 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/croitoruandreea/Desktop/VVSS-labs/Docs/Lab01/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82B7372-8EAD-8547-BC78-5DE929492666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="15960" windowHeight="18080" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Export Summary" sheetId="1" r:id="rId4"/>
-    <sheet name="Requirements Phase Defects" sheetId="2" r:id="rId5"/>
-    <sheet name="Architect. Design Phase Defects" sheetId="3" r:id="rId6"/>
-    <sheet name="Coding Phase Defects" sheetId="4" r:id="rId7"/>
-    <sheet name="Tool-basedCodeAnalysis" sheetId="5" r:id="rId8"/>
+    <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Requirements Phase Defects" sheetId="2" r:id="rId2"/>
+    <sheet name="Architect. Design Phase Defects" sheetId="3" r:id="rId3"/>
+    <sheet name="Coding Phase Defects" sheetId="4" r:id="rId4"/>
+    <sheet name="Tool-basedCodeAnalysis" sheetId="5" r:id="rId5"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="97">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -295,7 +317,7 @@
   <si>
     <r>
       <rPr>
-        <i val="1"/>
+        <i/>
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
@@ -304,8 +326,8 @@
     </r>
     <r>
       <rPr>
-        <b val="1"/>
-        <i val="1"/>
+        <b/>
+        <i/>
         <sz val="11"/>
         <color indexed="8"/>
         <rFont val="Calibri"/>
@@ -329,12 +351,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="0" formatCode="General"/>
-    <numFmt numFmtId="59" formatCode="dd.mm.yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -351,51 +372,54 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <u val="single"/>
+      <u/>
       <sz val="12"/>
       <color indexed="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="12"/>
       <color indexed="12"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="9"/>
       <color indexed="15"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="1"/>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -613,185 +637,134 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="59">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="58">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="5" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="8" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="6" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="6" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="6" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="7" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="7" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="7" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="49" fontId="7" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -800,32 +773,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ff5e88b1"/>
-      <rgbColor rgb="ffeef3f4"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ff000080"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffc00000"/>
-      <rgbColor rgb="ffe5dfec"/>
-      <rgbColor rgb="fffde9d9"/>
-      <rgbColor rgb="ffd2dae4"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FF5E88B1"/>
+      <rgbColor rgb="FFEEF3F4"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FFC00000"/>
+      <rgbColor rgb="FFE5DFEC"/>
+      <rgbColor rgb="FFFDE9D9"/>
+      <rgbColor rgb="FFD2DAE4"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
@@ -841,15 +867,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Screenshot 2026-03-15 at 14.26.29.png" descr="Screenshot 2026-03-15 at 14.26.29.png"/>
+        <xdr:cNvPr id="2" name="Screenshot 2026-03-15 at 14.26.29.png" descr="Screenshot 2026-03-15 at 14.26.29.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst/>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -875,7 +905,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -891,15 +921,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Screenshot 2026-03-15 at 14.29.55.png" descr="Screenshot 2026-03-15 at 14.29.55.png"/>
+        <xdr:cNvPr id="4" name="Screenshot 2026-03-15 at 14.29.55.png" descr="Screenshot 2026-03-15 at 14.29.55.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst/>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -925,7 +959,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
@@ -941,15 +975,19 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 1" descr="Picture 1"/>
+        <xdr:cNvPr id="6" name="Picture 1" descr="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst/>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -975,7 +1013,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
     <a:clrScheme name="Office Theme 2007 - 2010">
       <a:dk1>
@@ -1101,7 +1139,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1110,7 +1148,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1119,7 +1157,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="20000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1193,7 +1231,7 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+          <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
             <a:srgbClr val="000000">
               <a:alpha val="35000"/>
             </a:srgbClr>
@@ -1201,7 +1239,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1219,7 +1257,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1248,7 +1286,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1273,7 +1311,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1298,7 +1336,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1323,7 +1361,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1348,7 +1386,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1373,7 +1411,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1398,7 +1436,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1423,7 +1461,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1448,7 +1486,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1461,9 +1499,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -1478,7 +1522,7 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw blurRad="38100" dist="20000" dir="5400000" rotWithShape="0">
             <a:srgbClr val="000000">
               <a:alpha val="38000"/>
             </a:srgbClr>
@@ -1486,7 +1530,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1504,7 +1548,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1529,7 +1573,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1554,7 +1598,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1579,7 +1623,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1604,7 +1648,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1629,7 +1673,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1654,7 +1698,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1679,7 +1723,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1704,7 +1748,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1729,7 +1773,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1742,9 +1786,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1758,7 +1808,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1776,7 +1826,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1805,7 +1855,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1830,7 +1880,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1855,7 +1905,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1880,7 +1930,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1905,7 +1955,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1930,7 +1980,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1955,7 +2005,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1980,7 +2030,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2005,7 +2055,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -2018,103 +2068,111 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B3:D16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="13" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="4" width="30.5547" customWidth="1"/>
+    <col min="2" max="4" width="30.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" ht="0.05" customHeight="1">
-      <c r="B3" t="s" s="1">
+    <row r="3" spans="2:4" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C3"/>
-      <c r="D3"/>
-    </row>
-    <row r="7">
-      <c r="B7" t="s" s="2">
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+    </row>
+    <row r="7" spans="2:4" ht="19" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C7" t="s" s="2">
+      <c r="C7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D7" t="s" s="2">
+      <c r="D7" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" t="s" s="3">
+    <row r="9" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="4"/>
-      <c r="C10" t="s" s="4">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D10" t="s" s="5">
+      <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" t="s" s="3">
+    <row r="11" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="4"/>
-      <c r="C12" t="s" s="4">
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D12" t="s" s="5">
+      <c r="D12" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" t="s" s="3">
+    <row r="13" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B13" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="4"/>
-      <c r="C14" t="s" s="4">
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D14" t="s" s="5">
+      <c r="D14" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" t="s" s="3">
+    <row r="15" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B15" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="4"/>
-      <c r="C16" t="s" s="4">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="2:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D16" t="s" s="5">
+      <c r="D16" s="4" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2123,469 +2181,471 @@
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D10" location="'Requirements Phase Defects'!R1C1" tooltip="" display="Requirements Phase Defects"/>
-    <hyperlink ref="D12" location="'Architect. Design Phase Defects'!R1C1" tooltip="" display="Architect. Design Phase Defects"/>
-    <hyperlink ref="D14" location="'Coding Phase Defects'!R1C1" tooltip="" display="Coding Phase Defects"/>
-    <hyperlink ref="D16" location="'Tool-basedCodeAnalysis'!R1C1" tooltip="" display="Tool-basedCodeAnalysis"/>
+    <hyperlink ref="D10" location="'Requirements Phase Defects'!R1C1" display="Requirements Phase Defects" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D12" location="'Architect. Design Phase Defects'!R1C1" display="Architect. Design Phase Defects" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D14" location="'Coding Phase Defects'!R1C1" display="Coding Phase Defects" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D16" location="'Tool-basedCodeAnalysis'!R1C1" display="Tool-basedCodeAnalysis" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.3516" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.3516" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.85156" style="6" customWidth="1"/>
-    <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.85156" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="5" customWidth="1"/>
+    <col min="3" max="4" width="16.33203125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="5" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="21" style="5" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="5" customWidth="1"/>
+    <col min="11" max="11" width="8.83203125" style="5" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="7"/>
-      <c r="B1" t="s" s="8">
+    <row r="1" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" t="s" s="11">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" t="s" s="13">
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+    </row>
+    <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+      <c r="B2" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="15"/>
-      <c r="I2" t="s" s="16">
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s" s="16">
+      <c r="J2" s="11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
-      <c r="H3" t="s" s="16">
+    <row r="3" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s" s="16">
+      <c r="I3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="18">
+      <c r="J3" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" t="s" s="19">
+    <row r="4" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s" s="20">
+      <c r="D4" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="10"/>
-      <c r="H4" t="s" s="16">
+      <c r="E4" s="43"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s" s="16">
+      <c r="I4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" t="s" s="19">
+    <row r="5" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s" s="23">
+      <c r="D5" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
-      <c r="H5" t="s" s="16">
+      <c r="E5" s="46"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" s="25"/>
-      <c r="C6" t="s" s="26">
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s" s="27">
+      <c r="D6" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" t="s" s="26">
+      <c r="E6" s="37"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="36">
         <v>46096</v>
       </c>
-      <c r="E7" s="28"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" t="s" s="32">
+      <c r="E7" s="37"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9"/>
+      <c r="B9" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="32">
+      <c r="C9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s" s="32">
+      <c r="D9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E9" t="s" s="33">
+      <c r="E9" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" ht="65.55" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="18">
+      <c r="F9" s="15"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" spans="1:10" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9"/>
+      <c r="B10" s="13">
         <v>1</v>
       </c>
-      <c r="C10" t="s" s="34">
+      <c r="C10" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D10" t="s" s="34">
+      <c r="D10" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E10" t="s" s="35">
+      <c r="E10" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" ht="52.55" customHeight="1">
-      <c r="A11" s="10"/>
-      <c r="B11" s="18">
-        <f>B10+1</f>
+      <c r="F10" s="15"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9"/>
+      <c r="B11" s="13">
+        <f t="shared" ref="B11:B25" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" t="s" s="34">
+      <c r="C11" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D11" t="s" s="34">
+      <c r="D11" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E11" t="s" s="35">
+      <c r="E11" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="22"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" ht="65.55" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="18">
-        <f>B11+1</f>
+      <c r="F11" s="15"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+    </row>
+    <row r="12" spans="1:10" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9"/>
+      <c r="B12" s="13">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" t="s" s="34">
+      <c r="C12" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D12" t="s" s="34">
+      <c r="D12" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E12" t="s" s="35">
+      <c r="E12" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" ht="13.55" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="18">
-        <f>B12+1</f>
+      <c r="F12" s="15"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9"/>
+      <c r="B13" s="13">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" ht="13.55" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="18">
-        <f>B13+1</f>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9"/>
+      <c r="B14" s="13">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" ht="13.55" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="18">
-        <f>B14+1</f>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9"/>
+      <c r="B15" s="13">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" ht="13.55" customHeight="1">
-      <c r="A16" s="10"/>
-      <c r="B16" s="18">
-        <f>B15+1</f>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9"/>
+      <c r="B16" s="13">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" ht="13.55" customHeight="1">
-      <c r="A17" s="10"/>
-      <c r="B17" s="18">
-        <f>B16+1</f>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9"/>
+      <c r="B17" s="13">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" ht="13.55" customHeight="1">
-      <c r="A18" s="10"/>
-      <c r="B18" s="18">
-        <f>B17+1</f>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="9"/>
+      <c r="B18" s="13">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" ht="13.55" customHeight="1">
-      <c r="A19" s="10"/>
-      <c r="B19" s="18">
-        <f>B18+1</f>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9"/>
+      <c r="B19" s="13">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row r="20" ht="13.55" customHeight="1">
-      <c r="A20" s="10"/>
-      <c r="B20" s="18">
-        <f>B19+1</f>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+    </row>
+    <row r="20" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9"/>
+      <c r="B20" s="13">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-    </row>
-    <row r="21" ht="13.55" customHeight="1">
-      <c r="A21" s="10"/>
-      <c r="B21" s="18">
-        <f>B20+1</f>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+    </row>
+    <row r="21" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="9"/>
+      <c r="B21" s="13">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-    </row>
-    <row r="22" ht="13.55" customHeight="1">
-      <c r="A22" s="10"/>
-      <c r="B22" s="18">
-        <f>B21+1</f>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+    </row>
+    <row r="22" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9"/>
+      <c r="B22" s="13">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23" ht="13.55" customHeight="1">
-      <c r="A23" s="10"/>
-      <c r="B23" s="18">
-        <f>B22+1</f>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+    </row>
+    <row r="23" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9"/>
+      <c r="B23" s="13">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row r="24" ht="13.55" customHeight="1">
-      <c r="A24" s="10"/>
-      <c r="B24" s="18">
-        <f>B23+1</f>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+    </row>
+    <row r="24" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="9"/>
+      <c r="B24" s="13">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" ht="13.55" customHeight="1">
-      <c r="A25" s="10"/>
-      <c r="B25" s="18">
-        <f>B24+1</f>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+    </row>
+    <row r="25" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9"/>
+      <c r="B25" s="13">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" ht="13.55" customHeight="1">
-      <c r="A26" s="9"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" ht="13.55" customHeight="1">
-      <c r="A27" s="9"/>
-      <c r="B27" s="10"/>
-      <c r="C27" t="s" s="39">
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+    </row>
+    <row r="26" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="8"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+    </row>
+    <row r="27" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="8"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="40"/>
-      <c r="E27" t="s" s="34">
+      <c r="D27" s="28"/>
+      <c r="E27" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F27" s="22"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2597,7 +2657,7 @@
     <mergeCell ref="D5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2606,475 +2666,475 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="41" customWidth="1"/>
-    <col min="2" max="2" width="12.3516" style="41" customWidth="1"/>
-    <col min="3" max="4" width="16.3516" style="41" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="41" customWidth="1"/>
-    <col min="6" max="8" width="8.85156" style="41" customWidth="1"/>
-    <col min="9" max="9" width="22.1719" style="41" customWidth="1"/>
-    <col min="10" max="10" width="8.85156" style="41" customWidth="1"/>
-    <col min="11" max="16384" width="8.85156" style="41" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="5" customWidth="1"/>
+    <col min="3" max="4" width="16.33203125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="5" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="22.1640625" style="5" customWidth="1"/>
+    <col min="10" max="11" width="8.83203125" style="5" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="7"/>
-      <c r="B1" t="s" s="8">
+    <row r="1" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" t="s" s="11">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" t="s" s="13">
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+    </row>
+    <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+      <c r="B2" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="15"/>
-      <c r="I2" t="s" s="16">
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s" s="16">
+      <c r="J2" s="11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
-      <c r="H3" t="s" s="16">
+    <row r="3" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s" s="16">
+      <c r="I3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="18">
+      <c r="J3" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" t="s" s="42">
+    <row r="4" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s" s="43">
+      <c r="D4" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="44"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="10"/>
-      <c r="H4" t="s" s="16">
+      <c r="E4" s="48"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s" s="16">
+      <c r="I4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" t="s" s="42">
+    <row r="5" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s" s="45">
+      <c r="D5" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
-      <c r="H5" t="s" s="16">
+      <c r="E5" s="50"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" s="25"/>
-      <c r="C6" t="s" s="26">
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s" s="27">
+      <c r="D6" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" t="s" s="26">
+      <c r="E6" s="37"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="36">
         <v>46096</v>
       </c>
-      <c r="E7" s="28"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" t="s" s="32">
+      <c r="E7" s="37"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9"/>
+      <c r="B9" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="32">
+      <c r="C9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s" s="32">
+      <c r="D9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E9" t="s" s="32">
+      <c r="E9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" ht="78.55" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="18">
+      <c r="F9" s="15"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" spans="1:10" ht="78.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9"/>
+      <c r="B10" s="13">
         <v>1</v>
       </c>
-      <c r="C10" t="s" s="34">
+      <c r="C10" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D10" t="s" s="35">
+      <c r="D10" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E10" t="s" s="35">
+      <c r="E10" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" ht="52.55" customHeight="1">
-      <c r="A11" s="10"/>
-      <c r="B11" s="18">
-        <f>B10+1</f>
+      <c r="F10" s="15"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9"/>
+      <c r="B11" s="13">
+        <f t="shared" ref="B11:B26" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" t="s" s="34">
+      <c r="C11" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D11" t="s" s="35">
+      <c r="D11" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E11" t="s" s="35">
+      <c r="E11" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="22"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" ht="39.55" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="18">
-        <f>B11+1</f>
+      <c r="F11" s="15"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+    </row>
+    <row r="12" spans="1:10" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9"/>
+      <c r="B12" s="13">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" t="s" s="34">
+      <c r="C12" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D12" t="s" s="34">
+      <c r="D12" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E12" t="s" s="35">
+      <c r="E12" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" ht="13.55" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="18">
-        <f>B12+1</f>
+      <c r="F12" s="15"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9"/>
+      <c r="B13" s="13">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" ht="13.55" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="18">
-        <f>B13+1</f>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9"/>
+      <c r="B14" s="13">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" ht="13.55" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="18">
-        <f>B14+1</f>
+      <c r="C14" s="24"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9"/>
+      <c r="B15" s="13">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" ht="13.55" customHeight="1">
-      <c r="A16" s="10"/>
-      <c r="B16" s="18">
-        <f>B15+1</f>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9"/>
+      <c r="B16" s="13">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" ht="13.55" customHeight="1">
-      <c r="A17" s="10"/>
-      <c r="B17" s="18">
-        <f>B16+1</f>
+      <c r="C16" s="24"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9"/>
+      <c r="B17" s="13">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="36"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" ht="13.55" customHeight="1">
-      <c r="A18" s="10"/>
-      <c r="B18" s="18">
-        <f>B17+1</f>
+      <c r="C17" s="24"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="9"/>
+      <c r="B18" s="13">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" ht="13.55" customHeight="1">
-      <c r="A19" s="10"/>
-      <c r="B19" s="18">
-        <f>B18+1</f>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9"/>
+      <c r="B19" s="13">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="36"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row r="20" ht="13.55" customHeight="1">
-      <c r="A20" s="10"/>
-      <c r="B20" s="18">
-        <f>B19+1</f>
+      <c r="C19" s="24"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+    </row>
+    <row r="20" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9"/>
+      <c r="B20" s="13">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-    </row>
-    <row r="21" ht="13.55" customHeight="1">
-      <c r="A21" s="10"/>
-      <c r="B21" s="18">
-        <f>B20+1</f>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+    </row>
+    <row r="21" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="9"/>
+      <c r="B21" s="13">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-    </row>
-    <row r="22" ht="13.55" customHeight="1">
-      <c r="A22" s="10"/>
-      <c r="B22" s="18">
-        <f>B21+1</f>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+    </row>
+    <row r="22" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9"/>
+      <c r="B22" s="13">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23" ht="13.55" customHeight="1">
-      <c r="A23" s="10"/>
-      <c r="B23" s="18">
-        <f>B22+1</f>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+    </row>
+    <row r="23" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9"/>
+      <c r="B23" s="13">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row r="24" ht="13.55" customHeight="1">
-      <c r="A24" s="10"/>
-      <c r="B24" s="18">
-        <f>B23+1</f>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+    </row>
+    <row r="24" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="9"/>
+      <c r="B24" s="13">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" ht="13.55" customHeight="1">
-      <c r="A25" s="10"/>
-      <c r="B25" s="18">
-        <f>B24+1</f>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+    </row>
+    <row r="25" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9"/>
+      <c r="B25" s="13">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" ht="13.55" customHeight="1">
-      <c r="A26" s="10"/>
-      <c r="B26" s="18">
-        <f>B25+1</f>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+    </row>
+    <row r="26" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="9"/>
+      <c r="B26" s="13">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="37"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" ht="13.55" customHeight="1">
-      <c r="A27" s="9"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28" ht="13.55" customHeight="1">
-      <c r="A28" s="9"/>
-      <c r="B28" s="10"/>
-      <c r="C28" t="s" s="39">
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+    </row>
+    <row r="27" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="8"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+    </row>
+    <row r="28" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="8"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="40"/>
-      <c r="E28" t="s" s="34">
+      <c r="D28" s="28"/>
+      <c r="E28" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F28" s="22"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3086,7 +3146,7 @@
     <mergeCell ref="D5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -3095,346 +3155,356 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M16"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="47" customWidth="1"/>
-    <col min="2" max="2" width="12.3516" style="47" customWidth="1"/>
-    <col min="3" max="3" width="16.3516" style="47" customWidth="1"/>
-    <col min="4" max="4" width="18" style="47" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="47" customWidth="1"/>
-    <col min="6" max="8" width="8.85156" style="47" customWidth="1"/>
-    <col min="9" max="9" width="26.6719" style="47" customWidth="1"/>
-    <col min="10" max="13" width="8.85156" style="47" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="47" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18" style="5" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="5" customWidth="1"/>
+    <col min="6" max="8" width="8.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="5" customWidth="1"/>
+    <col min="10" max="14" width="8.83203125" style="5" customWidth="1"/>
+    <col min="15" max="16384" width="8.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="7"/>
-      <c r="B1" t="s" s="8">
+    <row r="1" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" t="s" s="11">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-    </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" t="s" s="13">
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+    </row>
+    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+      <c r="B2" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="15"/>
-      <c r="I2" t="s" s="16">
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s" s="16">
+      <c r="J2" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="22"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
-      <c r="H3" t="s" s="16">
+      <c r="K2" s="15"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" t="s" s="48">
+      <c r="I3" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="10">
+        <v>232</v>
+      </c>
+      <c r="K3" s="15"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+    </row>
+    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s" s="49">
+      <c r="D4" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="10"/>
-      <c r="H4" t="s" s="16">
+      <c r="E4" s="52"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" t="s" s="48">
+      <c r="I4" s="58" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="10">
+        <v>232</v>
+      </c>
+      <c r="K4" s="15"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+    </row>
+    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s" s="51">
+      <c r="D5" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="52"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
-      <c r="H5" t="s" s="16">
+      <c r="E5" s="54"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" s="25"/>
-      <c r="C6" t="s" s="26">
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+    </row>
+    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s" s="27">
+      <c r="D6" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" t="s" s="26">
+      <c r="E6" s="37"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+    </row>
+    <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" t="s" s="32">
+      <c r="D7" s="57">
+        <v>46096</v>
+      </c>
+      <c r="E7" s="37"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+    </row>
+    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+    </row>
+    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9"/>
+      <c r="B9" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="32">
+      <c r="C9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s" s="32">
+      <c r="D9" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E9" t="s" s="32">
+      <c r="E9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" ht="64" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="18">
+      <c r="F9" s="15"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+    </row>
+    <row r="10" spans="1:13" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9"/>
+      <c r="B10" s="13">
         <v>1</v>
       </c>
-      <c r="C10" t="s" s="34">
+      <c r="C10" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s" s="35">
+      <c r="D10" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E10" t="s" s="35">
+      <c r="E10" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-    </row>
-    <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="10"/>
-      <c r="B11" s="18">
+      <c r="F10" s="15"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+    </row>
+    <row r="11" spans="1:13" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9"/>
+      <c r="B11" s="13">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" t="s" s="34">
+      <c r="C11" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="D11" t="s" s="34">
+      <c r="D11" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="E11" t="s" s="35">
+      <c r="E11" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="22"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="18">
+      <c r="F11" s="15"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+    </row>
+    <row r="12" spans="1:13" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9"/>
+      <c r="B12" s="13">
         <f>B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" t="s" s="34">
+      <c r="C12" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="D12" t="s" s="34">
+      <c r="D12" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="E12" t="s" s="35">
+      <c r="E12" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="18">
+      <c r="F12" s="15"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+    </row>
+    <row r="13" spans="1:13" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9"/>
+      <c r="B13" s="13">
         <f>B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" t="s" s="34">
+      <c r="C13" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="D13" t="s" s="35">
+      <c r="D13" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s" s="35">
+      <c r="E13" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="22"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-    </row>
-    <row r="14" ht="64" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="18">
+      <c r="F13" s="15"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+    </row>
+    <row r="14" spans="1:13" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9"/>
+      <c r="B14" s="13">
         <f>B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" t="s" s="34">
+      <c r="C14" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="D14" t="s" s="35">
+      <c r="D14" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="E14" t="s" s="35">
+      <c r="E14" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="F14" s="22"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="9"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" t="s" s="39">
+      <c r="F14" s="15"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+    </row>
+    <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+    </row>
+    <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="40"/>
-      <c r="E16" s="53">
+      <c r="D16" s="28"/>
+      <c r="E16" s="31">
         <v>1</v>
       </c>
-      <c r="F16" s="22"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3446,7 +3516,7 @@
     <mergeCell ref="D5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -3455,351 +3525,353 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.85156" style="54" customWidth="1"/>
-    <col min="2" max="2" width="12.3516" style="54" customWidth="1"/>
-    <col min="3" max="3" width="16.3516" style="54" customWidth="1"/>
-    <col min="4" max="4" width="18" style="54" customWidth="1"/>
-    <col min="5" max="5" width="23.8516" style="54" customWidth="1"/>
-    <col min="6" max="6" width="16.6719" style="54" customWidth="1"/>
-    <col min="7" max="8" width="8.85156" style="54" customWidth="1"/>
-    <col min="9" max="9" width="26.6719" style="54" customWidth="1"/>
-    <col min="10" max="10" width="8.85156" style="54" customWidth="1"/>
-    <col min="11" max="16384" width="8.85156" style="54" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="18" style="5" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.6640625" style="5" customWidth="1"/>
+    <col min="7" max="8" width="8.83203125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="5" customWidth="1"/>
+    <col min="10" max="11" width="8.83203125" style="5" customWidth="1"/>
+    <col min="12" max="16384" width="8.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="7"/>
-      <c r="B1" t="s" s="8">
+    <row r="1" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" t="s" s="11">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="9"/>
-      <c r="B2" t="s" s="13">
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+    </row>
+    <row r="2" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+      <c r="B2" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="15"/>
-      <c r="I2" t="s" s="16">
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s" s="16">
+      <c r="J2" s="11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
-      <c r="H3" t="s" s="16">
+    <row r="3" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s" s="16">
+      <c r="I3" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="18">
+      <c r="J3" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" t="s" s="48">
+    <row r="4" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="D4" t="s" s="49">
+      <c r="D4" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="10"/>
-      <c r="H4" t="s" s="16">
+      <c r="E4" s="52"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s" s="16">
+      <c r="I4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="13">
         <v>232</v>
       </c>
     </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" t="s" s="26">
+    <row r="5" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s" s="27">
+      <c r="D5" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="10"/>
-      <c r="H5" t="s" s="16">
+      <c r="E5" s="37"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" s="25"/>
-      <c r="C6" t="s" s="26">
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="10"/>
-      <c r="B9" t="s" s="32">
+      <c r="D6" s="57">
+        <v>46096</v>
+      </c>
+      <c r="E6" s="37"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+    </row>
+    <row r="8" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9"/>
+      <c r="B9" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="32">
+      <c r="C9" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="D9" t="s" s="32">
+      <c r="D9" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="E9" t="s" s="32">
+      <c r="E9" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="F9" t="s" s="32">
+      <c r="F9" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="G9" s="22"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" ht="112" customHeight="1">
-      <c r="A10" s="10"/>
-      <c r="B10" s="18">
+      <c r="G9" s="15"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+    </row>
+    <row r="10" spans="1:10" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9"/>
+      <c r="B10" s="13">
         <v>1</v>
       </c>
-      <c r="C10" t="s" s="34">
+      <c r="C10" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D10" t="s" s="35">
+      <c r="D10" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="E10" t="s" s="35">
+      <c r="E10" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="F10" t="s" s="35">
+      <c r="F10" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="G10" s="22"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="10"/>
-      <c r="B11" s="18">
+      <c r="G10" s="15"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" spans="1:10" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9"/>
+      <c r="B11" s="13">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" t="s" s="34">
+      <c r="C11" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D11" t="s" s="34">
+      <c r="D11" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="E11" t="s" s="16">
+      <c r="E11" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="F11" t="s" s="35">
+      <c r="F11" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="22"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="10"/>
-      <c r="B12" s="18">
+      <c r="G11" s="15"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+    </row>
+    <row r="12" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9"/>
+      <c r="B12" s="13">
         <f>B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" t="s" s="34">
+      <c r="C12" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D12" t="s" s="34">
+      <c r="D12" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="E12" t="s" s="35">
+      <c r="E12" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F12" t="s" s="35">
+      <c r="F12" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="22"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="18">
+      <c r="G12" s="15"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9"/>
+      <c r="B13" s="13">
         <f>B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" t="s" s="34">
+      <c r="C13" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D13" t="s" s="35">
+      <c r="D13" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="E13" t="s" s="35">
+      <c r="E13" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="F13" t="s" s="35">
+      <c r="F13" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="22"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="10"/>
-      <c r="B14" s="18">
+      <c r="G13" s="15"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+    </row>
+    <row r="14" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9"/>
+      <c r="B14" s="13">
         <f>B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" t="s" s="34">
+      <c r="C14" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="D14" t="s" s="35">
+      <c r="D14" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="E14" t="s" s="35">
+      <c r="E14" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="F14" t="s" s="35">
+      <c r="F14" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="22"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" ht="13.55" customHeight="1">
-      <c r="A15" s="9"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" ht="13.55" customHeight="1">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" t="s" s="55">
+      <c r="G14" s="15"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+    </row>
+    <row r="15" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="55" t="s">
         <v>96</v>
       </c>
       <c r="D16" s="56"/>
       <c r="E16" s="56"/>
-      <c r="F16" t="s" s="57">
+      <c r="F16" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" ht="13.55" customHeight="1">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" ht="13.55" customHeight="1">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" ht="13.55" customHeight="1">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3811,7 +3883,7 @@
     <mergeCell ref="D6:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>